<commit_message>
V5.63 veroboard: add C2/C3/C4 decoupling caps to layout + tracker
</commit_message>
<xml_diff>
--- a/bike_mate_veroboard.xlsx
+++ b/bike_mate_veroboard.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="265">
   <si>
     <t xml:space="preserve">Bike-Mate veroboard: parts (13 strips A-M x 30 holes)</t>
   </si>
@@ -280,6 +280,48 @@
     <t xml:space="preserve">Column 27: J = collector, K = base, L = emitter</t>
   </si>
   <si>
+    <t xml:space="preserve">C2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decoupling across SuperMini 5V/GND, close to header (K = 5V, J = GND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-47 uF electrolytic, 16 V or higher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulk on 5V rail. + lead to K5 (5V), - lead to J5 (GND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacitor (optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switched 12V rail near IRF4905 (B = switched 12V, E = GND). Shares hole E30 with W4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total parts</t>
   </si>
   <si>
@@ -337,9 +379,6 @@
     <t xml:space="preserve">W4</t>
   </si>
   <si>
-    <t xml:space="preserve">E30</t>
-  </si>
-  <si>
     <t xml:space="preserve">M30</t>
   </si>
   <si>
@@ -776,6 +815,9 @@
   </si>
   <si>
     <t xml:space="preserve">MP1584, Mini 360, USB charger, GPS, fan, OLED, buzzer, NTC, button and LED connect by wire to the pads; their footprints are not on the board.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2, C3 and C4 were added after the first layout (recommended extra capacitors). C4 is optional.</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO 2 and GPIO 9 are strapping pins and must be high at reset. Measure sleep current with ACC off (see veroboard.txt known issues).</t>
@@ -1204,7 +1246,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1637,41 +1679,119 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D20" s="5" t="n">
-        <f aca="false">SUM(D4:D18)</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+      <c r="B19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="5" t="n">
-        <f aca="false">COUNTIF(H4:H18,"Yes")</f>
+      <c r="F19" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <f aca="false">SUM(D4:D21)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <f aca="false">COUNTIF(H4:H21,"Yes")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <f aca="false">D20-D21</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
-        <v>87</v>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <f aca="false">D23-D24</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H4:H18" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H4:H21" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1701,7 +1821,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1715,82 +1835,82 @@
         <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">COUNTA(A4:A8)</f>
@@ -1824,32 +1944,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>15</v>
@@ -1857,13 +1977,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>15</v>
@@ -1871,13 +1991,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>15</v>
@@ -1885,13 +2005,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>15</v>
@@ -1899,13 +2019,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>15</v>
@@ -1913,13 +2033,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>15</v>
@@ -1927,13 +2047,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>15</v>
@@ -1941,13 +2061,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>15</v>
@@ -1955,13 +2075,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>15</v>
@@ -1969,13 +2089,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>15</v>
@@ -1983,13 +2103,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>15</v>
@@ -1997,13 +2117,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>15</v>
@@ -2011,13 +2131,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>15</v>
@@ -2025,13 +2145,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>15</v>
@@ -2039,13 +2159,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>15</v>
@@ -2053,13 +2173,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>15</v>
@@ -2067,13 +2187,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>15</v>
@@ -2081,13 +2201,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>15</v>
@@ -2095,13 +2215,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>15</v>
@@ -2109,13 +2229,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>15</v>
@@ -2123,13 +2243,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>15</v>
@@ -2137,13 +2257,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>15</v>
@@ -2151,13 +2271,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>15</v>
@@ -2165,7 +2285,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="C28" s="5" t="n">
         <f aca="false">COUNTA(A4:A26)</f>
@@ -2174,7 +2294,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="C29" s="5" t="n">
         <f aca="false">COUNTIF(D4:D26,"Yes")</f>
@@ -2214,32 +2334,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>8</v>
@@ -2247,13 +2367,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>8</v>
@@ -2261,13 +2381,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>1</v>
@@ -2275,7 +2395,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUM(D4:D6)</f>
@@ -2310,160 +2430,160 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -2492,18 +2612,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2511,7 +2631,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="C4" s="4"/>
     </row>
@@ -2520,7 +2640,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="C5" s="4"/>
     </row>
@@ -2529,7 +2649,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="C6" s="4"/>
     </row>
@@ -2538,7 +2658,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="C7" s="4"/>
     </row>
@@ -2547,7 +2667,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="C8" s="4"/>
     </row>
@@ -2556,7 +2676,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="C9" s="4"/>
     </row>
@@ -2565,7 +2685,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="C10" s="4"/>
     </row>
@@ -2574,7 +2694,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="C11" s="4"/>
     </row>
@@ -2583,7 +2703,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="C12" s="4"/>
     </row>
@@ -2592,13 +2712,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="C13" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="C15" s="7" t="n">
         <f aca="false">COUNTIF(C4:C13,"Yes")/COUNTA(A4:A13)</f>
@@ -2627,7 +2747,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -2635,47 +2755,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>250</v>
+        <v>263</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>